<commit_message>
added filter by name
</commit_message>
<xml_diff>
--- a/IngSoftware/propuesta/CasosDeTests/CasosTest-Agregar Producto en Pedido.xlsx
+++ b/IngSoftware/propuesta/CasosDeTests/CasosTest-Agregar Producto en Pedido.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rojas\source\TrabajoFinalAus\IngSoftware\propuesta\CasosDeTests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB567CE-90FD-4450-9FC8-8B075732C763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930910F3-CFBA-477A-88FD-F72B61173F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{F2043960-19A0-48A2-9953-7906032BD69C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{F2043960-19A0-48A2-9953-7906032BD69C}"/>
   </bookViews>
   <sheets>
     <sheet name="1A-CASO FELIZ" sheetId="4" r:id="rId1"/>
-    <sheet name="1B-FILTRO POR CAT" sheetId="1" r:id="rId2"/>
-    <sheet name="1C-CANTIDAD INVALIDA" sheetId="2" r:id="rId3"/>
+    <sheet name="1B_1A-FILTRO CATEGORIA" sheetId="1" r:id="rId2"/>
+    <sheet name="1B_1A1A-FILTRO SIN RESULTADOS" sheetId="7" r:id="rId3"/>
+    <sheet name="1C_5A-CANTIDAD INVALIDA" sheetId="2" r:id="rId4"/>
+    <sheet name="1D_5A-CANTIDAD NO DISPONIBLE" sheetId="5" r:id="rId5"/>
+    <sheet name="1E_5B-QUITAR DEL PEDIDO" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="59">
   <si>
     <t xml:space="preserve">MISSTORTAS </t>
   </si>
@@ -86,13 +89,6 @@
   </si>
   <si>
     <t>N/A</t>
-  </si>
-  <si>
-    <t>Se utiliza el filtro por Categoria y/o Nombre del producto y se agrega la cantidad de producto deseado.</t>
-  </si>
-  <si>
-    <t>Filtro = "Torta de chocolate"
-Cantidad=2</t>
   </si>
   <si>
     <t>Se agrega la cantidad solicitada al Pedido.</t>
@@ -111,24 +107,134 @@
     <t>Se previene el guardado de productos en el Pedido con cantidad invalida.</t>
   </si>
   <si>
-    <t>Agregar producto al pedido.</t>
-  </si>
-  <si>
     <t>1A</t>
   </si>
   <si>
-    <t>1B</t>
-  </si>
-  <si>
-    <t>Filtro = "Tortas"
+    <t xml:space="preserve">Filtro = "Torta de chocolate"
+</t>
+  </si>
+  <si>
+    <t>Cantidad=2</t>
+  </si>
+  <si>
+    <t>El Sistema emite un cartel indicando que la cantidad ingresada fue agregada al carrito con exito.</t>
+  </si>
+  <si>
+    <t>Se ingresa a la vista de Productos.</t>
+  </si>
+  <si>
+    <t>Se utiliza el filtro por  Nombre del producto.</t>
+  </si>
+  <si>
+    <t>Los Productos a la venta son filtrados basandose en la entrada del filtro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
 Cantidad=2</t>
   </si>
   <si>
-    <t>Filtro = "Torta de chocolate"
-Cantidad=Cantidad mayor a la disponible, negativa o decimal (flotante).</t>
-  </si>
-  <si>
-    <t>1C</t>
+    <t xml:space="preserve">Filtro = "Tortas"
+</t>
+  </si>
+  <si>
+    <t>Los Productos a la venta son filtrados segun Categoria utilizando la entrada del filtro.</t>
+  </si>
+  <si>
+    <t>Se utiliza el filtro por Categoria de producto.</t>
+  </si>
+  <si>
+    <t>Se ingresa la cantidad de producto deseada en el recuadro del mismo y se selecciona la opcion de 'Agregar'.</t>
+  </si>
+  <si>
+    <t>Se accede a la Grilla de productos donde se pueden visualizar los productos a las venta con los siguientes campos: Nombre, Descripcion y Precio por unidad de los Productos.
+Aquellos productos con cantidad nula, se indica que no hay Cantidad disponible.</t>
+  </si>
+  <si>
+    <t>El Sistema actualiza automaticamente el Pedido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro = "Brownie de Coco"
+</t>
+  </si>
+  <si>
+    <t>Los Productos a la venta son filtrados segun Nombre.</t>
+  </si>
+  <si>
+    <t>Se utiliza el filtro por Nombre de producto.</t>
+  </si>
+  <si>
+    <t>Se selecciona el campo para agregar cantidad deseada de Producto.</t>
+  </si>
+  <si>
+    <t>El Sistema previene la modificacion de Cantidades de Producto. 
+El sistema indica mediante una leyenda que no hay productos disponibles a la venta.
+El Sistema permite utilizar los filtros nuevamente.</t>
+  </si>
+  <si>
+    <t>El Sistema emite un cartel indicando que la cantidad ingresada no es valida.</t>
+  </si>
+  <si>
+    <t>Cantidad=Cantidad mayor a la disponible, negativa o decimal (flotante).</t>
+  </si>
+  <si>
+    <t>No se agregan productos no disponibles.</t>
+  </si>
+  <si>
+    <t>* Existe un Producto a la Venta llamado "Brownie de Coco" con 0 productos a la venta disponibles.</t>
+  </si>
+  <si>
+    <t>Agregar Producto al Carrito: Cantidad no disponible.</t>
+  </si>
+  <si>
+    <t>Agregar producto al pedido. Cantidad invalida.</t>
+  </si>
+  <si>
+    <t>Se ingresa la cantidad de producto a quitar en el recuadro del mismo y se selecciona la opcion de 'Quitar'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro = "Torta de Chocolate"
+</t>
+  </si>
+  <si>
+    <t>El Sistema actualiza automaticamente el Pedido.
+El pedido continua sin productos para agregar.</t>
+  </si>
+  <si>
+    <t>El Sistema actualiza automaticamente el Pedido.
+Se agregan dos "Torta de chocolate" al Pedido.</t>
+  </si>
+  <si>
+    <t>El Sistema emite un cartel indicando que la cantidad solicitada fue quitada con exito.</t>
+  </si>
+  <si>
+    <t>Cantidad=3</t>
+  </si>
+  <si>
+    <t>1E_5B</t>
+  </si>
+  <si>
+    <t>1C_5A</t>
+  </si>
+  <si>
+    <t>1D_5A</t>
+  </si>
+  <si>
+    <t>1B_1A</t>
+  </si>
+  <si>
+    <t>* No existen Productos a la venta disponibles.</t>
+  </si>
+  <si>
+    <t>Se utiliza el filtro.</t>
+  </si>
+  <si>
+    <t>Los Productos a la venta son filtrados.
+No aparecen productos disponibles.
+El Sistema permite modificar el filtro.</t>
+  </si>
+  <si>
+    <t>El Sistema actualiza automaticamente el Pedido.
+El pedido no posee Productos.</t>
   </si>
 </sst>
 </file>
@@ -170,7 +276,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -193,11 +299,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -236,11 +368,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="60">
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -526,6 +667,13 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -544,9 +692,494 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
@@ -747,51 +1380,102 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{80B857B2-7D9D-4007-B12C-B58F5CED5C78}" name="Table2312145" displayName="Table2312145" ref="A7:E9" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
-  <autoFilter ref="A7:E9" xr:uid="{F04FAE14-76F5-400B-AEB2-3DF683100792}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{80B857B2-7D9D-4007-B12C-B58F5CED5C78}" name="Table2312145" displayName="Table2312145" ref="A7:E11" totalsRowShown="0" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48" tableBorderDxfId="46" totalsRowBorderDxfId="45">
+  <autoFilter ref="A7:E11" xr:uid="{F04FAE14-76F5-400B-AEB2-3DF683100792}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{FBF0EF42-207A-47E5-86E6-8A26DC132C48}" name="Numero de Paso" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{19516019-03D9-4677-9A31-65A6983A6BCB}" name="Accion" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{CBF799B7-994E-4EDC-87A9-F18F6C48B6BF}" name="Entrada" dataDxfId="2">
+    <tableColumn id="1" xr3:uid="{FBF0EF42-207A-47E5-86E6-8A26DC132C48}" name="Numero de Paso" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{19516019-03D9-4677-9A31-65A6983A6BCB}" name="Accion" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{CBF799B7-994E-4EDC-87A9-F18F6C48B6BF}" name="Entrada" dataDxfId="42">
       <calculatedColumnFormula array="1">- Nombre = "Torta de Chocolate"
 - Cantidad = "1"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{F75F0653-D1F9-459A-9899-7386674724BA}" name="Resultados" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{1ADC1041-1ABA-46A5-A82B-7663C6F25156}" name="Comentarios" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{F75F0653-D1F9-459A-9899-7386674724BA}" name="Resultados" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{1ADC1041-1ABA-46A5-A82B-7663C6F25156}" name="Comentarios" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F04FAE14-76F5-400B-AEB2-3DF683100792}" name="Table231214" displayName="Table231214" ref="A7:E9" totalsRowShown="0" headerRowDxfId="29" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26" totalsRowBorderDxfId="25">
-  <autoFilter ref="A7:E9" xr:uid="{F04FAE14-76F5-400B-AEB2-3DF683100792}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F04FAE14-76F5-400B-AEB2-3DF683100792}" name="Table231214" displayName="Table231214" ref="A7:E11" totalsRowShown="0" headerRowDxfId="39" dataDxfId="37" headerRowBorderDxfId="38" tableBorderDxfId="36" totalsRowBorderDxfId="35">
+  <autoFilter ref="A7:E11" xr:uid="{F04FAE14-76F5-400B-AEB2-3DF683100792}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{62C5A2BA-2AC8-4F17-A2F4-523D8D2E2286}" name="Numero de Paso" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{81F5EF2F-48B0-4BCA-BC71-07832011EA9B}" name="Accion" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{C9DE965B-4D3E-4519-BFD4-7E2BB2E451A3}" name="Entrada" dataDxfId="22">
+    <tableColumn id="1" xr3:uid="{62C5A2BA-2AC8-4F17-A2F4-523D8D2E2286}" name="Numero de Paso" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{81F5EF2F-48B0-4BCA-BC71-07832011EA9B}" name="Accion" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{C9DE965B-4D3E-4519-BFD4-7E2BB2E451A3}" name="Entrada" dataDxfId="32">
       <calculatedColumnFormula array="1">- Nombre = "Torta de Chocolate"
 - Cantidad = "1"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B3B9EE5F-60BD-4C7E-A4F9-EB560384CEE3}" name="Resultados" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{E008D7C0-FA83-43A4-86D1-44543CB9B102}" name="Comentarios" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{B3B9EE5F-60BD-4C7E-A4F9-EB560384CEE3}" name="Resultados" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{E008D7C0-FA83-43A4-86D1-44543CB9B102}" name="Comentarios" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2125E6B1-F35F-4208-9A37-3E2BA691953D}" name="Table2312144" displayName="Table2312144" ref="A7:E9" totalsRowShown="0" headerRowDxfId="19" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16" totalsRowBorderDxfId="15">
-  <autoFilter ref="A7:E9" xr:uid="{2125E6B1-F35F-4208-9A37-3E2BA691953D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{84AB0003-42B4-408B-8045-1CBC961208FF}" name="Table2312147" displayName="Table2312147" ref="A7:E9" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="A7:E9" xr:uid="{F04FAE14-76F5-400B-AEB2-3DF683100792}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{3F1A1CEF-AA43-491E-A5D9-DD8513C0895C}" name="Numero de Paso" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{7A59EFFF-8331-4BEC-B997-34E9103C703C}" name="Accion" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{55B3047B-ED64-4484-A204-A5E315735382}" name="Entrada" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{E9B8C6DD-311F-4682-9900-B81A2A05C9A3}" name="Numero de Paso" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{90036664-D653-477F-B4BD-E75E837F7D88}" name="Accion" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{C2AEDB9E-B026-46F3-A3FA-D110B75D0D8B}" name="Entrada" dataDxfId="2">
       <calculatedColumnFormula array="1">- Nombre = "Torta de Chocolate"
 - Cantidad = "1"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{448CA4FB-B720-43F8-B6B4-3341A8C6D516}" name="Resultados" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{F51923D8-58E8-4423-829C-C1B937464D04}" name="Comentarios" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{36114D38-4ADD-4167-9385-34ABB75531AA}" name="Resultados" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{06E865D8-D69A-4CAE-95C0-A1E60C4E49EA}" name="Comentarios" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2125E6B1-F35F-4208-9A37-3E2BA691953D}" name="Table2312144" displayName="Table2312144" ref="A7:E10" totalsRowShown="0" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58" tableBorderDxfId="56" totalsRowBorderDxfId="55">
+  <autoFilter ref="A7:E10" xr:uid="{2125E6B1-F35F-4208-9A37-3E2BA691953D}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{3F1A1CEF-AA43-491E-A5D9-DD8513C0895C}" name="Numero de Paso" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{7A59EFFF-8331-4BEC-B997-34E9103C703C}" name="Accion" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{55B3047B-ED64-4484-A204-A5E315735382}" name="Entrada" dataDxfId="52">
+      <calculatedColumnFormula array="1">- Nombre = "Torta de Chocolate"
+- Cantidad = "1"</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{448CA4FB-B720-43F8-B6B4-3341A8C6D516}" name="Resultados" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{F51923D8-58E8-4423-829C-C1B937464D04}" name="Comentarios" dataDxfId="50"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DCA6C85E-E705-481D-8423-D0390E3E9724}" name="Table2312143" displayName="Table2312143" ref="A7:E10" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" headerRowBorderDxfId="26" tableBorderDxfId="27" totalsRowBorderDxfId="25">
+  <autoFilter ref="A7:E10" xr:uid="{DCA6C85E-E705-481D-8423-D0390E3E9724}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{D9863D52-6750-4A02-A4BD-7E68039B95DD}" name="Numero de Paso" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{F6C7199D-2D02-4B57-BCFA-D0E554EBC2FA}" name="Accion" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{49A73671-90BE-4610-8C20-2B657A380F56}" name="Entrada" dataDxfId="22">
+      <calculatedColumnFormula array="1">- Nombre = "Torta de Chocolate"
+- Cantidad = "1"</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{FDF8C58F-A066-4343-B50D-C480878830A8}" name="Resultados" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{6EA0A753-4D85-43B7-9525-E6CE84245494}" name="Comentarios" dataDxfId="20"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A422D139-8549-4C43-8D5E-2A24CCE7C55E}" name="Table2312146" displayName="Table2312146" ref="A7:E15" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" headerRowBorderDxfId="16" tableBorderDxfId="17" totalsRowBorderDxfId="15">
+  <autoFilter ref="A7:E15" xr:uid="{A422D139-8549-4C43-8D5E-2A24CCE7C55E}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{D7EFC504-95C0-41DE-A9FA-6002EB668967}" name="Numero de Paso" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{77FC9B66-3302-461B-8532-99E411F921D5}" name="Accion" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{0D24EBDD-4F22-4B9A-BDFF-D8476752BC18}" name="Entrada" dataDxfId="12">
+      <calculatedColumnFormula array="1">- Nombre = "Torta de Chocolate"
+- Cantidad = "1"</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{9A8A3240-6308-42DF-A2DC-2993542532ED}" name="Resultados" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{B57E253A-06B2-46B2-8203-D976230AF629}" name="Comentarios" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1114,12 +1798,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D40990-3EF8-4A91-BA83-F92025DC4E76}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="38.5703125" customWidth="1"/>
     <col min="3" max="3" width="36.42578125" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="36.28515625" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1144,7 +1828,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1153,7 +1837,7 @@
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>4</v>
@@ -1168,13 +1852,13 @@
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1210,31 +1894,65 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+    <row r="8" spans="1:5" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
         <v>1</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>2</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="10"/>
+    </row>
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>3</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="16"/>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>4</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
+      <c r="D11" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1253,12 +1971,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8A9C318-9DC9-4AF6-BEE7-254C73036C02}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="38.5703125" customWidth="1"/>
     <col min="3" max="3" width="36.42578125" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="30.85546875" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1283,7 +2001,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1292,7 +2010,7 @@
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>4</v>
@@ -1307,13 +2025,13 @@
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1349,31 +2067,65 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+    <row r="8" spans="1:5" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
         <v>1</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>2</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="16"/>
+    </row>
+    <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>3</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="10"/>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>4</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
+      <c r="D11" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1391,17 +2143,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59C847A6-FC16-4936-9447-6D37FCA3926A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E89023-56B7-43A4-9266-AC57470FEB60}">
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="4" width="29.5703125" customWidth="1"/>
-    <col min="5" max="5" width="33.140625" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" customWidth="1"/>
+    <col min="4" max="4" width="30.85546875" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1422,7 +2174,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1431,7 +2183,7 @@
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>4</v>
@@ -1440,19 +2192,19 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1488,31 +2240,584 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+    <row r="8" spans="1:5" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
         <v>1</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>2</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:E6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59C847A6-FC16-4936-9447-6D37FCA3926A}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="37" customWidth="1"/>
+    <col min="3" max="4" width="40.42578125" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>19</v>
       </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
+        <v>1</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>2</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>36</v>
+      </c>
       <c r="C9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="16"/>
+    </row>
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>3</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:E6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E08FDC77-494E-42A2-B536-431E3A2CD1D7}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" customWidth="1"/>
+    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.85546875" customWidth="1"/>
+    <col min="4" max="4" width="37.140625" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
+        <v>1</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
+      <c r="D8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>2</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="16"/>
+    </row>
+    <row r="10" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>3</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:E6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9C2014C-CA21-44A2-9B46-F04E4C19FFB1}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="33.28515625" customWidth="1"/>
+    <col min="3" max="3" width="29.140625" customWidth="1"/>
+    <col min="4" max="4" width="60.7109375" customWidth="1"/>
+    <col min="5" max="5" width="41.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
+        <v>1</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>2</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="16"/>
+    </row>
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>3</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="10"/>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>4</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="10"/>
+    </row>
+    <row r="12" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>5</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="16"/>
+    </row>
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>6</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" s="10"/>
+    </row>
+    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="14">
+        <v>7</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="10"/>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>8</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>